<commit_message>
Sync Ocean Mist price to R230 and stop overwriting spreadsheet on build.
Price edits must be saved in the GitHub repo folder, then committed and pushed to update the live site.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/press-ons.xlsx
+++ b/data/press-ons.xlsx
@@ -1,41 +1,78 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/97b461c14d8dbcca/Documents/Cursor/Uniska Website/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_1C17020706397D6A2061021188D68B03A02C50A2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AEF44F0-3B18-4205-A98C-8E45713E0796}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Press-Ons" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>file</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>1. Blush Bloom.jpg</t>
+  </si>
+  <si>
+    <t>Blush Bloom</t>
+  </si>
+  <si>
+    <t>2. Soft Elegance.jpg</t>
+  </si>
+  <si>
+    <t>Soft Elegance</t>
+  </si>
+  <si>
+    <t>3. Ocean Mist.jpg</t>
+  </si>
+  <si>
+    <t>Ocean Mist</t>
+  </si>
+  <si>
+    <t>4. Classic French.jpg</t>
+  </si>
+  <si>
+    <t>Classic French</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +102,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,72 +441,74 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.796875" customWidth="1"/>
+    <col min="2" max="2" width="22.796875" customWidth="1"/>
+    <col min="3" max="3" width="12.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>file</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>price</v>
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>1. Blush Bloom.jpg</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Blush Bloom</v>
+    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
       </c>
       <c r="C2">
         <v>210</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2. Soft Elegance.jpg</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Soft Elegance</v>
+    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
       </c>
       <c r="C3">
         <v>210</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3. Ocean Mist.jpg</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Ocean Mist</v>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
       </c>
       <c r="C4">
-        <v>210</v>
+        <v>230</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>4. Classic French.jpg</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Classic French</v>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
       </c>
       <c r="C5">
         <v>210</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError sqref="A1:C3 A5:C5 A4:B4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>